<commit_message>
feature: change template for excel import
</commit_message>
<xml_diff>
--- a/public/Template.xlsx
+++ b/public/Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dennishadzialic/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://helsingborgsstad-my.sharepoint.com/personal/maria_sjodin_helsingborg_se/Documents/_Transparenta transporter/Sam/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B39895A0-D7A4-F040-9A3F-11BD7CE4F73A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F57CA36-3D1B-2A40-84DA-C0D9B6C49E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21460" yWindow="7220" windowWidth="28240" windowHeight="17240" xr2:uid="{B51409EB-5E58-264F-96A8-6EB089D89220}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15880" xr2:uid="{B51409EB-5E58-264F-96A8-6EB089D89220}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -78,6 +78,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos"/>
@@ -103,11 +109,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -125,8 +135,176 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>317500</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>355600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>546100</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>774700</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Bildobjekt 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8CAEE800-5520-DE0C-32C2-DB37045370F8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="317500" y="355600"/>
+          <a:ext cx="1473200" cy="1473200"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>812800</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="6134100" cy="2057400"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="textruta 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{237B7374-362F-01CE-2012-35D39722A719}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2057400" y="25400"/>
+          <a:ext cx="6134100" cy="2057400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1600" b="1"/>
+            <a:t>Rapportmall för att leverera öppen transportdata</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1600" b="1" baseline="0"/>
+            <a:t> till Sam</a:t>
+          </a:r>
+          <a:endParaRPr lang="sv-SE" sz="1600" b="1"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1200"/>
+            <a:t>Förklaring av kolumner</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1200" b="1"/>
+            <a:t>Orgnr</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1200" baseline="0"/>
+            <a:t> - Ditt företags organisationsnummer för att identifiera vem som har gjort en leverans</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1200" b="1" baseline="0"/>
+            <a:t>Levereras med </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1200" baseline="0"/>
+            <a:t>- ID för att identifiera en specifik tur, kan till exempel vara registreringsnummer för levererande lastbil</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1200" b="1" baseline="0"/>
+            <a:t>Till enhet </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1200" baseline="0"/>
+            <a:t>- ID för enheten som tar emot leveransen. Som ID används enhetens GLN-nummer. [Förteckning över GLN-nummer för Helsinborg stads enheter/leveransplatser]</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1200" b="1" baseline="0"/>
+            <a:t>Tidpunkt</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1200" baseline="0"/>
+            <a:t> - Ange tidpunkt när leveransen sker med år-månad-dag samt tidpunkt i tt:mm.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="sv-SE" sz="1200" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="sv-SE" sz="1200" baseline="0"/>
+            <a:t>Rapport levereras till kontaktperson utifrån överenskommet intervall.</a:t>
+          </a:r>
+          <a:endParaRPr lang="sv-SE" sz="1200"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-tema">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -442,57 +620,74 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{131C53F5-1A4E-424F-A97D-CDB99CE37B96}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" customWidth="1"/>
-    <col min="2" max="2" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.33203125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="24.5" customWidth="1"/>
+    <col min="3" max="3" width="47.33203125" customWidth="1"/>
+    <col min="4" max="4" width="19.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
+    <row r="1" spans="1:4" ht="83" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="2">
-        <v>7411244010</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>5</v>
-      </c>
+    <row r="2" spans="1:4" ht="83" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="3">
+      <c r="A3" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="5">
         <v>7411244010</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="6">
+        <v>7411244010</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>6</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>